<commit_message>
Refresh impact coverage + JV from Quest prod (1663 reps).
Re-pull sql/18 and sql/19 from data lake and regenerate impact_coverage_jv.xlsx.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/data/impact_coverage_jv.xlsx
+++ b/docs/data/impact_coverage_jv.xlsx
@@ -4706,9 +4706,6 @@
       <c r="K97" t="n">
         <v>0.1</v>
       </c>
-      <c r="L97" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -5008,9 +5005,6 @@
       <c r="K104" t="n">
         <v>0.1</v>
       </c>
-      <c r="L104" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11822,9 +11816,6 @@
       <c r="K259" t="n">
         <v>1</v>
       </c>
-      <c r="L259" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -16914,9 +16905,6 @@
       <c r="K375" t="n">
         <v>0</v>
       </c>
-      <c r="L375" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="376">
       <c r="A376" t="n">
@@ -30107,9 +30095,6 @@
       <c r="K676" t="n">
         <v>3.11</v>
       </c>
-      <c r="L676" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="677">
       <c r="A677" t="n">
@@ -30145,9 +30130,6 @@
       <c r="K677" t="n">
         <v>3.11</v>
       </c>
-      <c r="L677" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="678">
       <c r="A678" t="n">
@@ -32471,9 +32453,6 @@
       <c r="K730" t="n">
         <v>0</v>
       </c>
-      <c r="L730" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="731">
       <c r="A731" t="n">
@@ -42095,9 +42074,6 @@
       <c r="K949" t="n">
         <v>1.41</v>
       </c>
-      <c r="L949" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="950">
       <c r="A950" t="n">
@@ -42171,9 +42147,6 @@
       <c r="K951" t="n">
         <v>1.41</v>
       </c>
-      <c r="L951" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="952">
       <c r="A952" t="n">
@@ -42209,9 +42182,6 @@
       <c r="K952" t="n">
         <v>1.41</v>
       </c>
-      <c r="L952" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="953">
       <c r="A953" t="n">
@@ -42247,9 +42217,6 @@
       <c r="K953" t="n">
         <v>1.41</v>
       </c>
-      <c r="L953" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="954">
       <c r="A954" t="n">
@@ -42285,9 +42252,6 @@
       <c r="K954" t="n">
         <v>1.41</v>
       </c>
-      <c r="L954" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="955">
       <c r="A955" t="n">
@@ -42323,9 +42287,6 @@
       <c r="K955" t="n">
         <v>1.41</v>
       </c>
-      <c r="L955" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="956">
       <c r="A956" t="n">
@@ -42361,9 +42322,6 @@
       <c r="K956" t="n">
         <v>1.41</v>
       </c>
-      <c r="L956" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="957">
       <c r="A957" t="n">
@@ -64343,9 +64301,6 @@
       <c r="K1456" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="L1456" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="1457">
       <c r="A1457" t="n">
@@ -64494,9 +64449,6 @@
       </c>
       <c r="K1460" t="n">
         <v>0.07000000000000001</v>
-      </c>
-      <c r="L1460" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="1461">

</xml_diff>

<commit_message>
Refresh impact coverage + JV from Quest prod (2026-08-04).
Fresh sql/18 and sql/19 lake pull for Excel-only export; 1663 reps.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/data/impact_coverage_jv.xlsx
+++ b/docs/data/impact_coverage_jv.xlsx
@@ -828,6 +828,9 @@
       <c r="E9" t="n">
         <v>143</v>
       </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" t="n">
         <v>46590</v>
       </c>
@@ -4694,6 +4697,9 @@
       <c r="E97" t="n">
         <v>34</v>
       </c>
+      <c r="F97" t="n">
+        <v>0</v>
+      </c>
       <c r="H97" t="n">
         <v>21898.8</v>
       </c>
@@ -4993,6 +4999,9 @@
       <c r="E104" t="n">
         <v>37</v>
       </c>
+      <c r="F104" t="n">
+        <v>0</v>
+      </c>
       <c r="H104" t="n">
         <v>25775</v>
       </c>
@@ -11804,6 +11813,9 @@
       <c r="E259" t="n">
         <v>124</v>
       </c>
+      <c r="F259" t="n">
+        <v>0</v>
+      </c>
       <c r="H259" t="n">
         <v>21857.6</v>
       </c>
@@ -11839,6 +11851,9 @@
       <c r="E260" t="n">
         <v>111</v>
       </c>
+      <c r="F260" t="n">
+        <v>0</v>
+      </c>
       <c r="H260" t="n">
         <v>9830.799999999999</v>
       </c>
@@ -16893,6 +16908,9 @@
       <c r="E375" t="n">
         <v>94</v>
       </c>
+      <c r="F375" t="n">
+        <v>0</v>
+      </c>
       <c r="H375" t="n">
         <v>197531.2</v>
       </c>
@@ -17148,6 +17166,9 @@
       <c r="E381" t="n">
         <v>39</v>
       </c>
+      <c r="F381" t="n">
+        <v>0</v>
+      </c>
       <c r="H381" t="n">
         <v>64172</v>
       </c>
@@ -17362,6 +17383,9 @@
       <c r="E386" t="n">
         <v>64</v>
       </c>
+      <c r="F386" t="n">
+        <v>0</v>
+      </c>
       <c r="H386" t="n">
         <v>38378.2</v>
       </c>
@@ -19292,6 +19316,9 @@
       <c r="E430" t="n">
         <v>15</v>
       </c>
+      <c r="F430" t="n">
+        <v>0</v>
+      </c>
       <c r="H430" t="n">
         <v>0</v>
       </c>
@@ -19987,6 +20014,9 @@
       <c r="E446" t="n">
         <v>32</v>
       </c>
+      <c r="F446" t="n">
+        <v>0</v>
+      </c>
       <c r="H446" t="n">
         <v>132419.2</v>
       </c>
@@ -20814,6 +20844,9 @@
       <c r="E465" t="n">
         <v>118</v>
       </c>
+      <c r="F465" t="n">
+        <v>0</v>
+      </c>
       <c r="H465" t="n">
         <v>17616.2</v>
       </c>
@@ -27716,6 +27749,9 @@
       <c r="E622" t="n">
         <v>44</v>
       </c>
+      <c r="F622" t="n">
+        <v>0</v>
+      </c>
       <c r="H622" t="n">
         <v>0</v>
       </c>
@@ -30083,6 +30119,9 @@
       <c r="E676" t="n">
         <v>92</v>
       </c>
+      <c r="F676" t="n">
+        <v>0</v>
+      </c>
       <c r="H676" t="n">
         <v>478973.7</v>
       </c>
@@ -30118,6 +30157,9 @@
       <c r="E677" t="n">
         <v>125</v>
       </c>
+      <c r="F677" t="n">
+        <v>0</v>
+      </c>
       <c r="H677" t="n">
         <v>264332.8</v>
       </c>
@@ -32441,6 +32483,9 @@
       <c r="E730" t="n">
         <v>38</v>
       </c>
+      <c r="F730" t="n">
+        <v>0</v>
+      </c>
       <c r="H730" t="n">
         <v>242526.9</v>
       </c>
@@ -42062,6 +42107,9 @@
       <c r="E949" t="n">
         <v>40</v>
       </c>
+      <c r="F949" t="n">
+        <v>0</v>
+      </c>
       <c r="H949" t="n">
         <v>743376.3</v>
       </c>
@@ -42097,6 +42145,9 @@
       <c r="E950" t="n">
         <v>41</v>
       </c>
+      <c r="F950" t="n">
+        <v>0</v>
+      </c>
       <c r="H950" t="n">
         <v>389930.1</v>
       </c>
@@ -42135,6 +42186,9 @@
       <c r="E951" t="n">
         <v>41</v>
       </c>
+      <c r="F951" t="n">
+        <v>0</v>
+      </c>
       <c r="H951" t="n">
         <v>1297383.6</v>
       </c>
@@ -42170,6 +42224,9 @@
       <c r="E952" t="n">
         <v>37</v>
       </c>
+      <c r="F952" t="n">
+        <v>0</v>
+      </c>
       <c r="H952" t="n">
         <v>573973</v>
       </c>
@@ -42205,6 +42262,9 @@
       <c r="E953" t="n">
         <v>40</v>
       </c>
+      <c r="F953" t="n">
+        <v>0</v>
+      </c>
       <c r="H953" t="n">
         <v>495743.6</v>
       </c>
@@ -42240,6 +42300,9 @@
       <c r="E954" t="n">
         <v>39</v>
       </c>
+      <c r="F954" t="n">
+        <v>0</v>
+      </c>
       <c r="H954" t="n">
         <v>762680.7</v>
       </c>
@@ -42275,6 +42338,9 @@
       <c r="E955" t="n">
         <v>42</v>
       </c>
+      <c r="F955" t="n">
+        <v>0</v>
+      </c>
       <c r="H955" t="n">
         <v>815646.1</v>
       </c>
@@ -42310,6 +42376,9 @@
       <c r="E956" t="n">
         <v>34</v>
       </c>
+      <c r="F956" t="n">
+        <v>0</v>
+      </c>
       <c r="H956" t="n">
         <v>518943.6</v>
       </c>
@@ -64289,6 +64358,9 @@
       <c r="E1456" t="n">
         <v>39</v>
       </c>
+      <c r="F1456" t="n">
+        <v>0</v>
+      </c>
       <c r="H1456" t="n">
         <v>143970.9</v>
       </c>
@@ -64324,6 +64396,9 @@
       <c r="E1457" t="n">
         <v>14</v>
       </c>
+      <c r="F1457" t="n">
+        <v>0</v>
+      </c>
       <c r="H1457" t="n">
         <v>107441.1</v>
       </c>
@@ -64362,6 +64437,9 @@
       <c r="E1458" t="n">
         <v>6</v>
       </c>
+      <c r="F1458" t="n">
+        <v>0</v>
+      </c>
       <c r="H1458" t="n">
         <v>293315.6</v>
       </c>
@@ -64400,6 +64478,9 @@
       <c r="E1459" t="n">
         <v>5</v>
       </c>
+      <c r="F1459" t="n">
+        <v>0</v>
+      </c>
       <c r="H1459" t="n">
         <v>80370</v>
       </c>
@@ -64438,6 +64519,9 @@
       <c r="E1460" t="n">
         <v>6</v>
       </c>
+      <c r="F1460" t="n">
+        <v>0</v>
+      </c>
       <c r="H1460" t="n">
         <v>458270.9</v>
       </c>
@@ -64473,6 +64557,9 @@
       <c r="E1461" t="n">
         <v>31</v>
       </c>
+      <c r="F1461" t="n">
+        <v>0</v>
+      </c>
       <c r="H1461" t="n">
         <v>57279.5</v>
       </c>
@@ -64510,6 +64597,9 @@
       </c>
       <c r="E1462" t="n">
         <v>7</v>
+      </c>
+      <c r="F1462" t="n">
+        <v>0</v>
       </c>
       <c r="H1462" t="n">
         <v>322537.7</v>

</xml_diff>